<commit_message>
feat: update mock result reports with detailed SKU/GPU data
FX611H PR1 (Intel + RTX 50): 3 SKUs — AQ001 RTX5060, AQ002 RTX5070Ti, AQ003 RTX5060 lower CPU
FA401EA PR2 (AMD Strix Point iGPU): 3 SKUs — BQ001 RX890M, BQ002 RX880M, BQ003 RX860M
G513RM PR1 (AMD + RTX 40): 2 SKUs — HQ001 RTX4070, HQ002 RTX4060

SOW sheet now shows GPU sub-header row and separate columns per GPU SKU.
More realistic benchmark/FPS values reflecting GPU tier differences.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mock_results/FA401EA_PR2_Result_20260418.xlsx
+++ b/mock_results/FA401EA_PR2_Result_20260418.xlsx
@@ -176,13 +176,13 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -555,9 +555,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
@@ -619,7 +619,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>AMD Ryzen AI 300 (Strix Point)</t>
+          <t>AMD Ryzen AI 300 Series (Strix Point) — Zen5 + RDNA 3.5 iGPU</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -633,7 +633,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Windows 11 24H2</t>
+          <t>Windows 11 24H2 (Build 26100)</t>
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
@@ -691,7 +691,7 @@
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>BD / SKU</t>
+          <t>BD / 料號</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -706,73 +706,73 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Panel</t>
+          <t>Panel / RAM</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>FA401EA-BQ001</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Ryzen AI 9 HX 375</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>RX 890M (iGPU)</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>14" 2.8K 90Hz OLED</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Radeon RX 890M (iGPU, 16CU)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>14" 2.8K 90Hz OLED / 32GB LPDDR5X-7500</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>FA401EA-BQ002</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Ryzen AI 7 HX 360</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>RX 880M (iGPU)</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>14" FHD 144Hz</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Radeon RX 880M (iGPU, 12CU)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>14" 2.8K 90Hz OLED / 32GB LPDDR5X-7500</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>FA401EA-BQ003</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Ryzen AI 5 350</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>RX 860M (iGPU)</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>14" FHD 60Hz</t>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Ryzen AI 5 360</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Radeon RX 860M (iGPU, 8CU)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>14" FHD 60Hz IPS   / 16GB LPDDR5X-6400</t>
         </is>
       </c>
     </row>
@@ -800,186 +800,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>▶  SKU：FA401EA-BQ001   |   FA401EA-BQ002   |   FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Test Item</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ001</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ002</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Multi Median (pts)</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="n">
+          <t>Cinebench R23 30-loop — Multi-Core Median (pts)</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
         <v>24580</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="10" t="n">
         <v>21340</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="10" t="n">
         <v>15670</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Multi Max (pts)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
+          <t>Cinebench R23 30-loop — Multi-Core Max (pts)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
         <v>25120</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="10" t="n">
         <v>21890</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="10" t="n">
         <v>16120</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Multi Min (pts)</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
+          <t>Cinebench R23 30-loop — Multi-Core Min (pts)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>24010</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="10" t="n">
         <v>20820</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="10" t="n">
         <v>15240</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="10" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Single Median (pts)</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
+          <t>Cinebench R23 30-loop — Single-Core Median (pts)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>1756</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="10" t="n">
         <v>1698</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="10" t="n">
         <v>1542</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Single Max (pts)</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
+          <t>Cinebench R23 30-loop — Single-Core Max (pts)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
         <v>1789</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="10" t="n">
         <v>1728</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="10" t="n">
         <v>1572</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="10" t="n">
         <v>6</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 30-loop Single Min (pts)</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
+          <t>Cinebench R23 30-loop — Single-Core Min (pts)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
         <v>1721</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="10" t="n">
         <v>1668</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="10" t="n">
         <v>1510</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="10" t="n">
         <v>7</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Power Limit (W)</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
+          <t>Power Limit — Turbo Mode (W)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="10" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Power Limit — Standard Mode (W)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -992,174 +1011,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>▶  SKU：FA401EA-BQ001   |   FA401EA-BQ002   |   FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Test Item</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ001</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ002</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Fire Strike (score)</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="n">
+          <t>Fire Strike — Graphics Score</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
         <v>8920</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="10" t="n">
         <v>7650</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="10" t="n">
         <v>5230</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Fire Strike Extreme (score)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
+          <t>Fire Strike — Physics Score</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>14250</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>14180</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>9540</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Fire Strike Extreme — Graphics Score</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>4520</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D5" s="10" t="n">
         <v>3890</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E5" s="10" t="n">
         <v>2640</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Fire Strike Ultra (score)</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Fire Strike Ultra — Graphics Score</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>2450</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D6" s="10" t="n">
         <v>2110</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E6" s="10" t="n">
         <v>1430</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Time Spy (score)</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Time Spy — Graphics Score</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
         <v>5840</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D7" s="10" t="n">
         <v>5010</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E7" s="10" t="n">
         <v>3420</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Time Spy Extreme (score)</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Time Spy — CPU Score</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>5120</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>5090</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>3680</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Time Spy Extreme — Graphics Score</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
         <v>2890</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D9" s="10" t="n">
         <v>2480</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E9" s="10" t="n">
         <v>1690</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Port Royal (score)</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Speed Way (score)</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Port Royal — Score</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Speed Way — Score</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>DLSS Feature Test (DLSS 4 MFG)</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1172,52 +1278,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>▶  SKU：FA401EA-BQ001   |   FA401EA-BQ002   |   FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Test Item</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ001</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ002</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1225,18 +1331,18 @@
           <t>MobileMark 25 — Modern Office (min)</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="10" t="n">
         <v>534</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="10" t="n">
         <v>568</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="10" t="n">
         <v>612</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1244,57 +1350,133 @@
           <t>MobileMark 25 — Video Playback (min)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="10" t="n">
         <v>698</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="10" t="n">
         <v>734</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="10" t="n">
         <v>789</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>MobileMark 25 — Content Creation (min)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>468</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>498</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
           <t>PCMark 10 Battery — Modern Office (min)</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C6" s="10" t="n">
         <v>476</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D6" s="10" t="n">
         <v>508</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E6" s="10" t="n">
         <v>548</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>PCMark 10 Battery — Video Playback (min)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C7" s="10" t="n">
         <v>812</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D7" s="10" t="n">
         <v>848</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E7" s="10" t="n">
         <v>901</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Web Browsing (Edge / YouTube) (min)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>612</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>648</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Battery Capacity (Wh)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>73</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>73</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Charging Time: 0→100% (min)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1307,186 +1489,281 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>▶  SKU：FA401EA-BQ001   |   FA401EA-BQ002   |   FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Test Item</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ001</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ002</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>FA401EA-BQ003</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 Multi (pts)</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="n">
+          <t>Cinebench R23 — Multi-Core (pts)</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
         <v>24560</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="10" t="n">
         <v>21230</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="10" t="n">
         <v>15640</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R23 Single (pts)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
+          <t>Cinebench R23 — Single-Core (pts)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
         <v>1748</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="10" t="n">
         <v>1690</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="10" t="n">
         <v>1534</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R24 Multi (pts)</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
+          <t>Cinebench R24 — Multi-Core (pts)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>16320</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="10" t="n">
         <v>14150</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="10" t="n">
         <v>10420</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="10" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cinebench R24 Single (pts)</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
+          <t>Cinebench R24 — Single-Core (pts)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>1189</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="10" t="n">
         <v>1145</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="10" t="n">
         <v>1042</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>PCMark 10 Overall (score)</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
+          <t>Cinebench 2024 — Multi-Core (pts)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>1398</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>PCMark 10 — Overall (score)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
         <v>7456</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D8" s="10" t="n">
         <v>7123</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E8" s="10" t="n">
         <v>6780</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>PCMark 10 Productivity (score)</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>PCMark 10 — Productivity (score)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
         <v>8890</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D9" s="10" t="n">
         <v>8542</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E9" s="10" t="n">
         <v>8102</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>CrossMark Overall (score)</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>PCMark 10 — Digital Content Creation (score)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>9540</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>9180</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>8620</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CrossMark — Overall (score)</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
         <v>1856</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D11" s="10" t="n">
         <v>1798</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E11" s="10" t="n">
         <v>1645</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>CrossMark — Productivity (score)</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>1945</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>1882</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>3DMark CPU Profile — 1T (pts)</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>980</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>948</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>3DMark CPU Profile — Max Threads (pts)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>24480</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>21160</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>15580</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>